<commit_message>
chore: mise à jour du fichier de répartition du travail
</commit_message>
<xml_diff>
--- a/Documentation/repartitionDuTravailFestivalOrganisation.xlsx
+++ b/Documentation/repartitionDuTravailFestivalOrganisation.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\benja\Desktop\COURS\BTS_SIO_2\SLAM\POO\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\benja\source\repos\Festival_Organisateur\Documentation\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{FF348582-5D1F-4E4D-AE1B-9DB1836AFDDC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6C77BDCA-B9A3-4D93-B819-83CD4CF4D1E8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" xr2:uid="{A593C323-CC7B-4F13-A495-34FE018599DB}"/>
   </bookViews>
@@ -16,6 +16,7 @@
     <sheet name="Feuil1" sheetId="1" r:id="rId1"/>
   </sheets>
   <calcPr calcId="191029"/>
+  <fileRecoveryPr repairLoad="1"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -34,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="35" uniqueCount="26">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="43" uniqueCount="32">
   <si>
     <t>festival_organisateur</t>
   </si>
@@ -105,13 +106,31 @@
     <t>Contorle sécu ..</t>
   </si>
   <si>
-    <t>modifie le spermissions des roles</t>
-  </si>
-  <si>
     <t>R</t>
   </si>
   <si>
     <t xml:space="preserve">Tournoi </t>
+  </si>
+  <si>
+    <t>Tournoir, Joueur</t>
+  </si>
+  <si>
+    <t>Tournoi</t>
+  </si>
+  <si>
+    <t>Jeu, Espace</t>
+  </si>
+  <si>
+    <t>Espace, Plateforme</t>
+  </si>
+  <si>
+    <t>Voter, Plateforme, Jeu</t>
+  </si>
+  <si>
+    <t>Orgaisateur, role</t>
+  </si>
+  <si>
+    <t>modifie les permissions des roles</t>
   </si>
 </sst>
 </file>
@@ -135,7 +154,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="4">
+  <fills count="7">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -144,13 +163,31 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="9"/>
+        <fgColor theme="4"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="4"/>
+        <fgColor rgb="FFFFC000"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF00B050"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF7030A0"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -167,11 +204,14 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -529,7 +569,10 @@
       <c r="A6" t="s">
         <v>7</v>
       </c>
-      <c r="C6" s="3"/>
+      <c r="C6" s="2"/>
+      <c r="E6" t="s">
+        <v>25</v>
+      </c>
       <c r="F6" t="s">
         <v>19</v>
       </c>
@@ -538,34 +581,37 @@
       <c r="A7" t="s">
         <v>8</v>
       </c>
-      <c r="C7" s="3"/>
+      <c r="C7" s="2"/>
       <c r="F7" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A8" t="s">
         <v>9</v>
       </c>
-      <c r="C8" s="3"/>
+      <c r="C8" s="2"/>
+      <c r="E8" t="s">
+        <v>29</v>
+      </c>
       <c r="F8" t="s">
         <v>21</v>
       </c>
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A9" t="s">
+      <c r="A9" s="6" t="s">
         <v>10</v>
       </c>
-      <c r="C9" s="3"/>
+      <c r="C9" s="2"/>
       <c r="F9" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A10" t="s">
         <v>11</v>
       </c>
-      <c r="B10" s="2"/>
+      <c r="B10" s="5"/>
       <c r="F10" t="s">
         <v>21</v>
       </c>
@@ -574,19 +620,25 @@
       <c r="A11" t="s">
         <v>12</v>
       </c>
-      <c r="B11" s="2"/>
+      <c r="B11" s="5"/>
+      <c r="E11" t="s">
+        <v>11</v>
+      </c>
       <c r="F11" t="s">
         <v>21</v>
       </c>
       <c r="G11" t="s">
-        <v>23</v>
+        <v>31</v>
       </c>
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A12" t="s">
         <v>13</v>
       </c>
-      <c r="C12" s="3"/>
+      <c r="C12" s="2"/>
+      <c r="E12" t="s">
+        <v>28</v>
+      </c>
       <c r="F12" t="s">
         <v>21</v>
       </c>
@@ -595,7 +647,7 @@
       <c r="A13" t="s">
         <v>14</v>
       </c>
-      <c r="C13" s="3"/>
+      <c r="C13" s="2"/>
       <c r="F13" t="s">
         <v>21</v>
       </c>
@@ -604,7 +656,10 @@
       <c r="A14" t="s">
         <v>15</v>
       </c>
-      <c r="B14" s="2"/>
+      <c r="B14" s="5"/>
+      <c r="E14" t="s">
+        <v>26</v>
+      </c>
       <c r="F14" t="s">
         <v>21</v>
       </c>
@@ -613,16 +668,19 @@
       <c r="A15" t="s">
         <v>16</v>
       </c>
-      <c r="B15" s="2"/>
+      <c r="B15" s="5"/>
+      <c r="E15" t="s">
+        <v>15</v>
+      </c>
       <c r="F15" t="s">
         <v>21</v>
       </c>
     </row>
     <row r="16" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A16" t="s">
+      <c r="A16" s="3" t="s">
         <v>17</v>
       </c>
-      <c r="C16" s="3"/>
+      <c r="C16" s="2"/>
       <c r="F16" t="s">
         <v>21</v>
       </c>
@@ -631,16 +689,22 @@
       <c r="A17" t="s">
         <v>20</v>
       </c>
-      <c r="B17" s="2"/>
+      <c r="B17" s="5"/>
+      <c r="E17" t="s">
+        <v>30</v>
+      </c>
       <c r="F17" t="s">
         <v>22</v>
       </c>
     </row>
     <row r="18" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A18" t="s">
-        <v>25</v>
-      </c>
-      <c r="C18" s="3"/>
+      <c r="A18" s="4" t="s">
+        <v>24</v>
+      </c>
+      <c r="C18" s="2"/>
+      <c r="E18" t="s">
+        <v>27</v>
+      </c>
       <c r="F18" t="s">
         <v>21</v>
       </c>

</xml_diff>